<commit_message>
feature: complete customer management module
</commit_message>
<xml_diff>
--- a/docs/Task_Group_2.xlsx
+++ b/docs/Task_Group_2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Meterials\FPT\4. SUM26\PRJ301\PRJ301_SE2039_Group_2\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F418FDD6-4A76-4DA9-8AE0-2A680313A0F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6020890-E7D0-4FA6-8ED8-6D5DB91A0240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>AUTOWASHPRO - TEAM TASK REPORT</t>
   </si>
@@ -51,48 +51,9 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Login/Logout, CustomerDAO</t>
-  </si>
-  <si>
-    <t>Authentication, session creation, logout, DB integration</t>
-  </si>
-  <si>
     <t>Completed</t>
   </si>
   <si>
-    <t>Register, CustomerDAO</t>
-  </si>
-  <si>
-    <t>Registration, duplicate validation, account creation</t>
-  </si>
-  <si>
-    <t>Database, SQL, Dashboard, VehicleDAO</t>
-  </si>
-  <si>
-    <t>DB schema, SQL scripts, VehicleDAO, dashboard data</t>
-  </si>
-  <si>
-    <t>Landing, SignIn, SignUp, Dashboard UI, MVC Refactor, Session Control</t>
-  </si>
-  <si>
-    <t>Session Management</t>
-  </si>
-  <si>
-    <t>Authentication Module</t>
-  </si>
-  <si>
-    <t>Registration Module</t>
-  </si>
-  <si>
-    <t>Dashboard UI</t>
-  </si>
-  <si>
-    <t>Dashboard MVC Refactor</t>
-  </si>
-  <si>
-    <t>Vehicle Statistics</t>
-  </si>
-  <si>
     <t>Student's ID</t>
   </si>
   <si>
@@ -120,9 +81,6 @@
     <t>Lecturer: Thân Thị Ngọc Vân</t>
   </si>
   <si>
-    <t>Completed Features Summary</t>
-  </si>
-  <si>
     <t>Last Updated: 01/6/2026</t>
   </si>
   <si>
@@ -150,10 +108,16 @@
     <t>Semester: Summer 2026</t>
   </si>
   <si>
-    <t>Landing, SignIn, SignUp, Dashboard UI, MVC Refactor, Session Control, Git Merge &amp; Conflict Resolution</t>
-  </si>
-  <si>
     <t>Repository:</t>
+  </si>
+  <si>
+    <t>Booking Management Logic, BookingDAO, Booking Validation</t>
+  </si>
+  <si>
+    <t>Administration Module Development</t>
+  </si>
+  <si>
+    <t>Vehicle &amp; Customer Management Module</t>
   </si>
 </sst>
 </file>
@@ -214,7 +178,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -231,8 +195,14 @@
         <fgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -278,15 +248,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -317,7 +278,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -345,20 +306,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -377,27 +329,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -406,6 +349,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -715,7 +664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" customWidth="1"/>
@@ -731,47 +680,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="32"/>
+      <c r="A2" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="26"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="32"/>
+      <c r="A3" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="26"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" s="32"/>
+      <c r="A4" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="26"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
+      <c r="A5" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
       <c r="D5" s="6"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="32" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
+      <c r="A6" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
       <c r="D6" s="6"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -787,10 +736,10 @@
       <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="25"/>
+      <c r="D8" s="21"/>
       <c r="E8" s="1" t="s">
         <v>4</v>
       </c>
@@ -798,195 +747,144 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>1</v>
       </c>
-      <c r="B9" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="26" t="s">
+      <c r="B9" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="23"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="27"/>
-      <c r="E9" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>2</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="27"/>
-      <c r="E10" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="23"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>3</v>
       </c>
-      <c r="B11" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="27"/>
-      <c r="E11" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="23"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>4</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="29"/>
-      <c r="E12" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="23"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="11" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="30" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" s="30"/>
-      <c r="C13" s="18"/>
+      <c r="A13" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="24"/>
+      <c r="C13" s="15"/>
       <c r="D13" s="7"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="31" t="str">
+      <c r="A14" s="25" t="str">
         <f>HYPERLINK(
 "https://github.com/phanthanhhung03/PRJ301_SE2039_Group_2.git",
 "https://github.com/phanthanhhung03/PRJ301_SE2039_Group_2.git"
 )</f>
         <v>https://github.com/phanthanhhung03/PRJ301_SE2039_Group_2.git</v>
       </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="16"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="13"/>
     </row>
     <row r="15" spans="1:6" s="9" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D15" s="17"/>
-      <c r="E15" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="F15" s="23"/>
+      <c r="D15" s="14"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B16" s="20"/>
+      <c r="B16" s="17"/>
       <c r="C16" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="16" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="19"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F17" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="16"/>
+      <c r="C18" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="16"/>
+      <c r="C19" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="19"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" s="16"/>
       <c r="C20" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F20" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E21" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>8</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="14">
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="E15:F15"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>

</xml_diff>